<commit_message>
upload results for 8node
</commit_message>
<xml_diff>
--- a/8node_spain/output_a.xlsx
+++ b/8node_spain/output_a.xlsx
@@ -468,25 +468,25 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.0007453695651671155</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>3.124314937118485e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>2.92812984600686e-05</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>5.909527291198822e-05</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1.717374396212979e-05</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>1.709683671241951e-05</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>2.993518521391164e-05</v>
       </c>
     </row>
     <row r="3">
@@ -496,28 +496,28 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>0.0007453695651671155</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0003978386713523962</v>
+        <v>4.02632862762199e-05</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>0.0008032159041748662</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>2.938912668358327e-05</v>
       </c>
       <c r="G3" t="n">
-        <v>2.016951252558324</v>
+        <v>1.952896425232338</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2031221295889138</v>
+        <v>0.1737562465310059</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>3.464187232550856e-05</v>
       </c>
     </row>
     <row r="4">
@@ -527,28 +527,28 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>3.124314937118485e-05</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0003978386713523962</v>
+        <v>4.02632862762199e-05</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>3.027324278143338e-05</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>3.470562991878609e-05</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>0.2271459810476383</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>0.0002956702665441288</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>4.64932228287365e-05</v>
       </c>
     </row>
     <row r="5">
@@ -558,28 +558,28 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>2.92812984600686e-05</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.0008032159041748662</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>3.027324278143338e-05</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>3.071462194007691e-05</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>0.4780236433170759</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>0.04906883333578367</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>2.665764144200257e-05</v>
       </c>
     </row>
     <row r="6">
@@ -589,28 +589,28 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>5.909527291198822e-05</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>2.938912668358327e-05</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>3.470562991878609e-05</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>3.071462194007691e-05</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>0.05294379747915855</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1.875011854212714e-05</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>3.96704806195417e-05</v>
       </c>
     </row>
     <row r="7">
@@ -620,28 +620,28 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1.717374396212979e-05</v>
       </c>
       <c r="C7" t="n">
-        <v>2.016951252558324</v>
+        <v>1.952896425232338</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.2271459810476383</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>0.4780236433170759</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>0.05294379747915855</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>6.013041542290318e-05</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>0.003036729878819212</v>
       </c>
     </row>
     <row r="8">
@@ -651,28 +651,28 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1.709683671241951e-05</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2031221295889138</v>
+        <v>0.1737562465310059</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.0002956702665441288</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>0.04906883333578367</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1.875011854212714e-05</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>6.013041542290318e-05</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>9.226143337959834e-05</v>
       </c>
     </row>
     <row r="9">
@@ -682,25 +682,25 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>2.993518521391164e-05</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>3.464187232550856e-05</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>4.64932228287365e-05</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>2.665764144200257e-05</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>3.96704806195417e-05</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>0.003036729878819212</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>9.226143337959834e-05</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>

</xml_diff>